<commit_message>
## [v1.3.0] — 2026-06-11
### Añadido
- EC-DIS: Documento de Diseño (Arquitectura del Sistema) (V 1.0, G.Gargaglione)

### Modificado
- EC-SCM: Plan de Gestión de Configuraciones (V 2.2, G.Gargaglione)
- EC-SQA-PLN: Plan de SQA (V 1.1, G. Gargaglione)
- EC-SRC-PHP: Catálogo público de muebles con conexión dinámica a MariaDB (catalogo.php)
- EC-REQ: Especificación de requerimientos.

### Notas
- Tercer iteración
- Realizado el análisis de riesgos y agregados planes de contingencia y mitigación,
con énfasis en los riesgos "Factores personales" y "Falta de revisión entre pares".
- Agregado el requerimiento RF-10 (Ver detalle de mueble)
</commit_message>
<xml_diff>
--- a/docs/gestion/riesgos/EC-RSG-ANL_analisis_id_riesgos.xlsx
+++ b/docs/gestion/riesgos/EC-RSG-ANL_analisis_id_riesgos.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Control de versiones" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="42">
   <si>
     <t xml:space="preserve">Control de versiones del documento</t>
   </si>
@@ -50,6 +50,21 @@
     <t xml:space="preserve">Identificacion y analisis de los primeros riesgos detectados</t>
   </si>
   <si>
+    <t xml:space="preserve">2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G. Gargaglione</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Análisis de los riesgos, donde “Cambio de requerimientos” y “Retroalimentación” fueron los riesgos más importantes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nuevo análisis de riesgos, incorporación de planes de mitigación y contingencia. Eliminación de riesgos R03 y R04  “Falta de aptitud en lenguaje” y “Cambio de requerimientos durante el proyecto” ya que son relativos a la asignatura. Se aumentó el impacto y probabilidad de “Factores personales”. Disminuida la probabilidad de falta de retroalimentación.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Riesgo</t>
   </si>
   <si>
@@ -68,6 +83,12 @@
     <t xml:space="preserve">Factor</t>
   </si>
   <si>
+    <t xml:space="preserve">Plan de Contingencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plan de Mitigación</t>
+  </si>
+  <si>
     <t xml:space="preserve">R01</t>
   </si>
   <si>
@@ -80,6 +101,42 @@
     <t xml:space="preserve">Cronograma</t>
   </si>
   <si>
+    <t xml:space="preserve">Establecer fechas internas de entrega con anticipación a los plazos reales, y comunicar avances parciales al cliente de forma proactiva para mantener su confianza.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Si el retraso ocurre, notificar al cliente con la mayor anticipación posible, explicar el estado real del proyecto y </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">negociar un nuevo plazo</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">.</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">R02</t>
   </si>
   <si>
@@ -92,51 +149,164 @@
     <t xml:space="preserve">Personal</t>
   </si>
   <si>
-    <t xml:space="preserve">R03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cambio de requerimientos durante la ejecución del proyecto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si el cliente modifica lo que pidió originalmente, el equipo debe replanificar tareas, modificar módulos que ya estaban cerrados y, en muchos casos, rehacer parte del trabajo previo. Esto provoca demoras en el cronograma, genera conflictos sobre el alcance contratado, y obliga a renegociar plazos. Si los cambios son frecuentes o profundos, el proyecto puede entrar en una espiral donde nunca se logre estabilizar el alcance y la fecha de entrega se vuelve imposible de cumplir.</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Mantener la documentación y el código siempre actualizado en el repositorio para que cualquier integrante pueda retomar el trabajo sin depender del otro. </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Distribuir el conocimiento del proyecto entre ambos integrantes.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">R05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falta de retroalimentación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A pesar de avanzar en el proyecto, el cliente no ha dado una nueva "retroalimentación" para continuar con el desarrollo del proyecto, lo cual deja cierta incertidumbre sobre como proceder.</t>
   </si>
   <si>
     <t xml:space="preserve">Requisitos</t>
   </si>
   <si>
-    <t xml:space="preserve">R04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Falta de aptitud en herramientas / lenguaje</t>
-  </si>
-  <si>
-    <t xml:space="preserve">En caso de que haya problemas a la hora de usar cualquier tipo de metodología, herramienta, etc en el ambiente laboral pueden surgir problemas en la calidad de los entregables y/o un retraso en la entrega de los insumos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Experiencia y Capacidad</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avances/Retroalimentación</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A pesar de avanzar en el proyecto, el cliente no ha dado una nueva "retroalimentación" para continuar con el desarrollo del proyecto, lo cual deja cierta incertidumbre sobre como proceder.</t>
+    <t xml:space="preserve">R06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Falta de revisión entre pares</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Los entregables se presentan sin validación interna, </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">aumentando la probabilidad de errores no detectados.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">No bloquea la entrega pero reduce la calidad.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Proceso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Al inicio de cada iteración se definen fechas internas de entrega para cada parte, con un mínimo de 24 horas de anticipación al horario de clase. El estado de cada tarea se refleja en el tablero GitHub Projects y se comunica activamente entre los integrantes por Discord o WhatsApp.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Si un integrante no ha completado ni comunicado el estado de su parte con al menos </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">24 horas de anticipación al horario de clase</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, el otro integrante </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">queda habilitado para asumir esas tareas o presentar el trabajo con el alcance disponible</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Helvetica Neue"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, dejando constancia del motivo en el repositorio mediante un Issue con etiqueta scr.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="166" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
-    <numFmt numFmtId="168" formatCode="@"/>
-    <numFmt numFmtId="169" formatCode="0.00\ %"/>
-    <numFmt numFmtId="170" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="@"/>
+    <numFmt numFmtId="170" formatCode="0.00\ %"/>
+    <numFmt numFmtId="171" formatCode="General"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -193,7 +363,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,6 +374,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -242,7 +418,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
@@ -255,83 +431,83 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="15" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="15" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="15" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="15" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="15" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="15" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -344,7 +520,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -377,28 +553,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF8696B"/>
+          <fgColor rgb="FFE0E282"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFF8E983"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFA7F70"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB84"/>
+          <fgColor rgb="FFF8696B"/>
         </patternFill>
       </fill>
     </dxf>
@@ -467,7 +629,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla" displayName="Tabla" ref="A1:G6" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla" displayName="Tabla" ref="A1:G4" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <tableColumns count="7">
     <tableColumn id="1" name="Riesgo"/>
     <tableColumn id="2" name="Descripción"/>
@@ -502,71 +664,87 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="1" style="1" width="24.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="29.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="6" t="n">
         <v>46173</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="7" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
+    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>46182</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>46184</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -587,161 +765,172 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:I1048576"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="7" width="9.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="7" width="17.24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="7" width="64.85"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="8" width="13.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="9" width="10.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="7" width="14.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="7" width="8.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="9" width="9.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="9" width="17.24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="9" width="46.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="9" width="13.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="10" width="10.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="9" width="14.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="9" width="8.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="40.61"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40.05"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="B1" s="10" t="s">
+    <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F1" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="G1" s="10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" s="7" customFormat="true" ht="55.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="C1" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="D1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="E1" s="13" t="s">
         <v>16</v>
       </c>
+      <c r="F1" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" s="9" customFormat="true" ht="73.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>23</v>
+      </c>
       <c r="D2" s="15" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E2" s="16" t="n">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="G2" s="18" t="n">
         <f aca="false">PRODUCT(E2:F2,100)</f>
-        <v>17.5</v>
-      </c>
-    </row>
-    <row r="3" s="7" customFormat="true" ht="74.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>20</v>
+        <v>225</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="19" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" s="9" customFormat="true" ht="103.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>29</v>
       </c>
       <c r="D3" s="15" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="E3" s="16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>0.45</v>
+        <v>0.95</v>
       </c>
       <c r="G3" s="18" t="n">
         <f aca="false">PRODUCT(E3:F3,100)</f>
-        <v>135</v>
-      </c>
-    </row>
-    <row r="4" s="7" customFormat="true" ht="98.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>24</v>
+        <v>380</v>
+      </c>
+      <c r="H3" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="84.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>34</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E4" s="16" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="F4" s="17" t="n">
-        <v>0.55</v>
+        <v>0.01</v>
       </c>
       <c r="G4" s="18" t="n">
         <f aca="false">PRODUCT(E4:F4,100)</f>
-        <v>247.5</v>
-      </c>
-    </row>
-    <row r="5" s="7" customFormat="true" ht="50.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" s="19" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>29</v>
+        <v>3</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="99.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>39</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>2.6</v>
+        <v>3.5</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>0.5</v>
+        <v>0.95</v>
       </c>
       <c r="G5" s="18" t="n">
         <f aca="false">PRODUCT(E5:F5,100)</f>
-        <v>130</v>
-      </c>
-    </row>
-    <row r="6" s="7" customFormat="true" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="16" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="17" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="G6" s="18" t="n">
-        <f aca="false">PRODUCT(E6:F6,100)</f>
-        <v>270</v>
-      </c>
-    </row>
+        <v>332.5</v>
+      </c>
+      <c r="H5" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <conditionalFormatting sqref="G1:G1048576">
     <cfRule type="colorScale" priority="2">
@@ -766,11 +955,11 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:B6" type="none">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="A2:B5" type="none">
       <formula1>0</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="E2:G6" type="custom">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="true" showErrorMessage="false" showInputMessage="false" sqref="E2:G5" type="custom">
       <formula1>AND(ISNUMBER(E2),(NOT(OR(NOT(ISERROR(DATEVALUE(E2))), AND(ISNUMBER(E2), LEFT(CELL("format", E2))="D")))))</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>